<commit_message>
vault backup: 2026-06-25 18:19:09
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/马来西亚社媒采集预算_确定版_最高口径.xlsx
+++ b/公司项目/认知作战/马来西亚社媒采集预算_确定版_最高口径.xlsx
@@ -132,7 +132,7 @@
     <t>10TB，2TB 价格 3,282.51 元 × 5</t>
   </si>
   <si>
-    <t>按截图 SSD 2TB 价格乘 5</t>
+    <t>电商价格</t>
   </si>
   <si>
     <t>本地 HDD</t>
@@ -722,17 +722,16 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Microsoft YaHei"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="10"/>
       <name val="Microsoft YaHei"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1215,19 +1214,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1236,7 +1235,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1360,7 +1359,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1395,7 +1394,10 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1403,6 +1405,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2106,49 +2111,49 @@
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:8">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:8">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="14">
         <v>1662594.502</v>
       </c>
-      <c r="C3" s="14">
+      <c r="C3" s="15">
         <v>166.2594502</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="16" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:8">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="14">
         <v>1388562.502</v>
       </c>
-      <c r="C4" s="14">
+      <c r="C4" s="15">
         <v>138.8562502</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:8">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="14">
         <v>1249170.502</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="15">
         <v>124.9170502</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2180,7 +2185,7 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:8">
-      <c r="A8" s="4">
+      <c r="A8" s="17">
         <v>1</v>
       </c>
       <c r="B8" s="4" t="s">
@@ -2206,7 +2211,7 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:8">
-      <c r="A9" s="4">
+      <c r="A9" s="17">
         <v>2</v>
       </c>
       <c r="B9" s="4" t="s">
@@ -2232,7 +2237,7 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:8">
-      <c r="A10" s="4">
+      <c r="A10" s="17">
         <v>3</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -2258,7 +2263,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:8">
-      <c r="A11" s="4">
+      <c r="A11" s="17">
         <v>4</v>
       </c>
       <c r="B11" s="4" t="s">
@@ -2282,7 +2287,7 @@
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:8">
-      <c r="A12" s="4">
+      <c r="A12" s="17">
         <v>5</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -2308,7 +2313,7 @@
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:8">
-      <c r="A13" s="4">
+      <c r="A13" s="17">
         <v>6</v>
       </c>
       <c r="B13" s="4" t="s">
@@ -2332,7 +2337,7 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:8">
-      <c r="A14" s="4">
+      <c r="A14" s="17">
         <v>7</v>
       </c>
       <c r="B14" s="4" t="s">

</xml_diff>